<commit_message>
vat-knowledge/plants_abroad: MIRO-Eingangsmatrix (Vorsteuerseite) ergaenzt
Neues Tabellenblatt "MIRO_Eingang" in beiden Workbooks (EPDE 22 / EPROHA 11
Faelle) mit den erwarteten Eingangs-/Vorsteuer-Kennzeichen, abgeleitet aus der
in:-Seite von SAP_TAX_MAP.

- Vier Vorgaenge: ig. Erwerb (VE/VH/W5/EC/UR/BP/EP/LP/NP/IP), Inlandseinkauf
  (VD/V2/B7/IB/...), Reverse Charge (DC/RC/VI), Einfuhr Drittland (EUSt/EORI);
  Sonderfall eigene Ware ab Werk = not relevant
- Zwei Zusatz-Eingaben (Lieferantenland + eingehende Lieferung bewegt/ruhend),
  die die Verkaufsseite nicht hergibt und die ig. Erwerb vs. Inlandseinkauf
  entscheiden
- Hinweis-Blatt + README um MIRO-Logik und die offene Frage (automatisch vs.
  manuell, gemaess Workshop) erweitert

Alle in:-Codes gegen getSapCode(...,'buyer') validiert (W5/VD/EC/DC/B7/VI ·
VE/IB/RC/VH).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BMKbRkyEepa3uat53j1you
</commit_message>
<xml_diff>
--- a/vat-knowledge/plants_abroad/Matrix_erweitert_EPROHA.xlsx
+++ b/vat-knowledge/plants_abroad/Matrix_erweitert_EPROHA.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Matrix_EPROHA" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Hinweise" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MIRO_Eingang" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -39,7 +40,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -49,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="007A2E1F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -78,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -100,6 +106,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -581,58 +596,58 @@
           <t>Lager AT – WE Österreich (Inland)</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
         <is>
           <t>ATxxx</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -642,12 +657,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -660,58 +675,58 @@
           <t>Lager AT – WE Deutschland (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -721,12 +736,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -739,58 +754,58 @@
           <t>Lager AT – WE Italien (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -800,12 +815,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="P4" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -818,58 +833,58 @@
           <t>Lager DE – WE Deutschland (Inland)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>DS</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -879,12 +894,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="P5" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -897,58 +912,58 @@
           <t>Lager DE – WE Österreich (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>ATxxx</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -958,12 +973,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="O6" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="P6" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -976,58 +991,58 @@
           <t>Lager AT – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1037,12 +1052,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="O7" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="P7" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1055,58 +1070,58 @@
           <t>Lager AT – WE Liechtenstein (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1116,12 +1131,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
+      <c r="O8" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="P8" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1134,58 +1149,58 @@
           <t>Lager DE – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1195,12 +1210,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O9" s="3" t="inlineStr">
+      <c r="O9" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="P9" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1213,58 +1228,58 @@
           <t>Konsi-Lager CH – WE Schweiz (CH-Inland)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>‹Werk CH›</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1274,12 +1289,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="O10" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="P10" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1292,58 +1307,58 @@
           <t>Konsi-Lager CH – WE Liechtenstein (Schweizer MWST-Raum)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>‹Werk CH›</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M11" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1353,12 +1368,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="P11" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1371,58 +1386,58 @@
           <t>Strecke – Lieferant DE/EU – WE Österreich</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>ATxxx</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L12" s="9" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1432,12 +1447,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="P12" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1450,58 +1465,58 @@
           <t>Strecke – Lieferant DE/EU (≠DE) – WE Deutschland</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K13" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" s="9" t="inlineStr">
         <is>
           <t>DS</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M13" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1511,12 +1526,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr">
+      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="P13" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1529,58 +1544,58 @@
           <t>Strecke – Lieferant EU – WE Italien (Dreieck, BUKRS AT)</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -1590,12 +1605,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="P14" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1612,58 +1627,58 @@
           <t>Strecke – Lieferant EU – WE Ungarn (Dreieck, BUKRS AT)</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>HUxxx</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L15" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -1673,12 +1688,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O15" s="3" t="inlineStr">
+      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="P15" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1695,58 +1710,58 @@
           <t>Strecke – Lieferant DE – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="M16" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1756,12 +1771,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="O16" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="P16" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1778,58 +1793,58 @@
           <t>Strecke – Lieferant AT – WE Liechtenstein (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="M17" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1839,12 +1854,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O17" s="3" t="inlineStr">
+      <c r="O17" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P17" s="3" t="inlineStr">
+      <c r="P17" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1861,22 +1876,22 @@
           <t>Strecke EXW – Lieferant AT – WE Deutschland</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -1886,37 +1901,37 @@
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="M18" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -1926,12 +1941,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O18" s="3" t="inlineStr">
+      <c r="O18" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="P18" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1944,22 +1959,22 @@
           <t>Strecke EXW – Lieferant DE – WE Italien</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -1969,37 +1984,37 @@
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="M19" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -2009,12 +2024,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O19" s="3" t="inlineStr">
+      <c r="O19" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P19" s="3" t="inlineStr">
+      <c r="P19" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2027,22 +2042,22 @@
           <t>Strecke EXW – Lieferant DE – WE Deutschland (Inland)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2052,37 +2067,37 @@
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L20" s="9" t="inlineStr">
         <is>
           <t>DS</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="M20" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -2092,12 +2107,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr">
+      <c r="O20" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P20" s="3" t="inlineStr">
+      <c r="P20" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2110,22 +2125,22 @@
           <t>Strecke EXW – Lieferant IT (ohne EPROHA-Reg) – WE Slowenien</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2135,37 +2150,37 @@
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K21" s="8" t="inlineStr">
         <is>
           <t>SIxxx</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="L21" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="M21" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -2175,12 +2190,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O21" s="3" t="inlineStr">
+      <c r="O21" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P21" s="3" t="inlineStr">
+      <c r="P21" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2197,58 +2212,58 @@
           <t>Ausfuhr AT → CH (DAP/EXW, Kunde verzollt)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L22" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="M22" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2258,12 +2273,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O22" s="3" t="inlineStr">
+      <c r="O22" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="P22" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2280,58 +2295,58 @@
           <t>Ausfuhr AT → LI (DAP/EXW, Kunde verzollt)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="K23" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="L23" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="M23" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2341,12 +2356,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O23" s="3" t="inlineStr">
+      <c r="O23" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P23" s="3" t="inlineStr">
+      <c r="P23" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2363,58 +2378,58 @@
           <t>Ausfuhr DE → CH (über DE-Reg)</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="J24" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K24" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L24" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="M24" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2424,12 +2439,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O24" s="3" t="inlineStr">
+      <c r="O24" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="P24" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2446,58 +2461,58 @@
           <t>CH-Inland DDP – EPROHA CH-registriert – WE Schweiz</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>CH-Reg (CH+LI)</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J25" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K25" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="M25" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -2507,12 +2522,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O25" s="3" t="inlineStr">
+      <c r="O25" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="P25" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2529,58 +2544,58 @@
           <t>CH-Reg → WE Liechtenstein (Schweizer MWST-Raum, DDP)</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>CH-Reg (CH+LI)</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L26" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="M26" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -2590,12 +2605,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O26" s="3" t="inlineStr">
+      <c r="O26" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P26" s="3" t="inlineStr">
+      <c r="P26" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2612,58 +2627,58 @@
           <t>Ausfuhr AT → GB (DAP/EXW, Post-Brexit)</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K27" s="8" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="L27" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="M27" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2673,12 +2688,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O27" s="3" t="inlineStr">
+      <c r="O27" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P27" s="3" t="inlineStr">
+      <c r="P27" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2695,58 +2710,58 @@
           <t>Lager AT – WE Großbritannien (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K28" s="8" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L28" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="M28" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2756,12 +2771,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr">
+      <c r="O28" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="P28" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -2774,58 +2789,58 @@
           <t>Lager DE – WE Großbritannien (Ausfuhr über DE-Reg)</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K29" s="8" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L29" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="M29" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2835,12 +2850,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr">
+      <c r="O29" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P29" s="3" t="inlineStr">
+      <c r="P29" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -2853,58 +2868,58 @@
           <t>Dreieck – Lieferant Deutschland → EPROHA(AT) → WE Italien (Art. 141)</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="K30" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="M30" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -2914,12 +2929,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr">
+      <c r="O30" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="P30" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2936,58 +2951,58 @@
           <t>Dreieck – Lieferant Frankreich → EPROHA(AT) → WE Ungarn (Art. 141)</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J31" s="8" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="K31" s="8" t="inlineStr">
         <is>
           <t>HUxxx</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L31" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="M31" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -2997,12 +3012,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O31" s="3" t="inlineStr">
+      <c r="O31" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P31" s="3" t="inlineStr">
+      <c r="P31" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3019,58 +3034,58 @@
           <t>Drop-Ship – Kunde AT (legt fremde EU-UID vor) – Warenempfänger DE</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr"/>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="8" t="inlineStr">
         <is>
           <t>Kunde-UID (≠AT)</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K32" s="8" t="inlineStr">
         <is>
           <t>DE(Kunde AT)xxx</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L32" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="M32" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -3080,12 +3095,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O32" s="3" t="inlineStr">
+      <c r="O32" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P32" s="3" t="inlineStr">
+      <c r="P32" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3102,58 +3117,58 @@
           <t>Drop-Ship – Kunde AT (KEINE fremde UID) – Warenempfänger DE</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>BUKRS AT</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="K33" s="8" t="inlineStr">
         <is>
           <t>DE(Kunde AT)xxx</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L33" s="9" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr">
+      <c r="M33" s="8" t="inlineStr">
         <is>
           <t>Inland AT 20%</t>
         </is>
@@ -3163,12 +3178,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O33" s="3" t="inlineStr">
+      <c r="O33" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P33" s="3" t="inlineStr">
+      <c r="P33" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3185,58 +3200,58 @@
           <t>Drop-Ship – Kunde DE – Warenempfänger IT (Reihen-/Dreiecksgeschäft)</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr"/>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="8" t="inlineStr">
         <is>
           <t>AT (Ansässigkeit)</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K34" s="8" t="inlineStr">
         <is>
           <t>DE(Kunde)xxx</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="L34" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="M34" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung / Dreieck</t>
         </is>
@@ -3246,12 +3261,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O34" s="3" t="inlineStr">
+      <c r="O34" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P34" s="3" t="inlineStr">
+      <c r="P34" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3268,58 +3283,58 @@
           <t>Drop-Ship – Kunde CH (Drittland) – Warenempfänger SK (Ware bleibt EU)</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr"/>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>AT (Ansässigkeit)</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
         <is>
           <t>SK</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr">
+      <c r="K35" s="8" t="inlineStr">
         <is>
           <t>CH(Kunde)xxx</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L35" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M35" s="3" t="inlineStr">
+      <c r="M35" s="8" t="inlineStr">
         <is>
           <t>ig. Reihengeschäft (kein Export)</t>
         </is>
@@ -3329,12 +3344,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O35" s="3" t="inlineStr">
+      <c r="O35" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P35" s="3" t="inlineStr">
+      <c r="P35" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3356,7 +3371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3447,6 +3462,643 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>MIRO-Eingangsblatt</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Zweites Prinzip: die Eingangs-/Vorsteuerseite (MIRO). Blatt „MIRO_Eingang" leitet je Einkaufsfall das erwartete Eingangs-Kennzeichen ab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>MIRO — 4 Vorgänge</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>1) ig. Erwerb (eingehende Lieferung BEWEGT → Ankunftsland, Selbstveranlagung VE/VH/W5/EC/UR/BP/EP/LP/NP/IP, netto 0). 2) Inlandseinkauf (eingehende Lieferung RUHEND → Lieferant weist lokale MwSt aus, Vorsteuer VD/V2/B7/…). 3) Reverse Charge (DE §13b→DC, AT→RC, IT→VI). 4) Einfuhr Drittland (EUSt über EORI, kein Tabellen-MWSKZ). Sonderfall: eigene Ware ab Werk = kein Vorsteuervorgang (not relevant).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>MIRO — zwei Zusatz-Eingaben</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Anders als die Verkaufsseite braucht MIRO: (a) das LIEFERANTENLAND und (b) ob die EINGEHENDE Lieferung BEWEGT oder RUHEND ist. Genau das entscheidet zwischen ig. Erwerb (z. B. W5) und Inlandseinkauf (z. B. B7) — dieselbe Transportzuordnungs-Abhängigkeit wie oben.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>MIRO — offene Klärung</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Der Workshop hat MIRO als teils MANUELL markiert („steuerliches Abgangsland in der MIRO-Buchung korrekt pflegen"). Vor Automatisierung mit dem SAP-Team klären, ob die Findung MIRO automatisch ermitteln soll oder ob es ein manuell gepflegter Schritt bleibt.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Einkaufsfall</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>BUKRS</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Lieferantenland</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>eingehende Lieferung</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Waren-/Ankunftsland</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Erwerber-UID (BUKRS)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>tax code Miro</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Vorgang (Info)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Hinweis</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant DE → Ware nach AT</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>bewegt</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>ATU36513402</t>
+        </is>
+      </c>
+      <c r="G2" s="9" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>ig. Erwerb (Selbstveranlagung)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>ig. Erwerb AT (VE), netto 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant IT → Ware nach AT</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>IT</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>bewegt</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>ATU36513402</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>ig. Erwerb (Selbstveranlagung)</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>ig. Erwerb AT (VE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant FR → Ware nach DE (wir DE-registriert)</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>bewegt</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>DE248554278</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>ig. Erwerb (Selbstveranlagung)</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>ig. Erwerb DE über DE-UID (VH)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant AT → AT-Inlandslieferung an uns</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>ruhend</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>ATU36513402</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Inlandseinkauf (Vorsteuer)</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>20% AT-Vorsteuer V2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant DE → DE-Inlandslieferung an uns</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>ruhend</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>DE248554278</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Inlandseinkauf (Vorsteuer)</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>19% DE-Vorsteuer VD</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant CH → CH-Inlandslieferung (wir CH-registriert)</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>ruhend</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>CHE-113.857.016 MWST</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>IB</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Inlandseinkauf (Vorsteuer)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>8,1% CH-Vorsteuer IB</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant LI → LI-Inlandslieferung (Schweizer MWST-Raum)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>ruhend</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>CHE-113.857.016 MWST</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>IB</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>Inlandseinkauf (Vorsteuer)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>8,1% Vorsteuer IB – LI über CH-Registrierung</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>AT Werklieferung/Leistung mit Reverse Charge</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>ruhend</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>ATU36513402</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>Reverse Charge</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>AT-RC (§19 UStG) → Eingang RC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant CH → Einfuhr nach AT</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Einfuhr</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>EORI (keine UID)</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>EUSt / EORI (kein MWSKZ)</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>Einfuhr Drittland</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>EUSt über EORI, als Vorsteuer abziehbar – kein Tabellen-MWSKZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Lieferant GB → Einfuhr nach AT</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Einfuhr</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>EORI (keine UID)</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>EUSt / EORI (kein MWSKZ)</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>Einfuhr Drittland</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>EUSt über EORI (Post-Brexit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Eigene Ware ab AT-Lager (Direktlieferung)</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>entfällt</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>not relevant</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>kein Vorsteuervorgang</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>kein Vorsteuervorgang</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
plants_abroad: MIRO-Zeile fuer EXW-Strecke AT->DE (Verkauf AF -> Eingang V2)
Explizite MIRO_Eingang-Zeile fuer den Fall "Strecke EXW - Lieferant AT - WE
Deutschland": EPROHAs Verkauf ist die bewegte ig. Lieferung AT->DE (AF), die
eingehende Vorlieferung Lieferant(AT)->EPROHA ist folglich ruhend in AT ->
AT-Inlandseinkauf -> Vorsteuer V2. Verknuepft mit der Verkaufszeile, damit der
Zusammenhang Ausgang AF <-> Eingang V2 direkt dokumentiert ist.

EPROHA MIRO_Eingang: 11 -> 12 Faelle.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BMKbRkyEepa3uat53j1you
</commit_message>
<xml_diff>
--- a/vat-knowledge/plants_abroad/Matrix_erweitert_EPROHA.xlsx
+++ b/vat-knowledge/plants_abroad/Matrix_erweitert_EPROHA.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -106,6 +106,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -596,58 +605,58 @@
           <t>Lager AT – WE Österreich (Inland)</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr"/>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
         <is>
           <t>ATxxx</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -657,12 +666,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="O2" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="P2" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -675,58 +684,58 @@
           <t>Lager AT – WE Deutschland (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr"/>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -736,12 +745,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -754,58 +763,58 @@
           <t>Lager AT – WE Italien (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr"/>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="M4" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -815,12 +824,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O4" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="P4" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -833,58 +842,58 @@
           <t>Lager DE – WE Deutschland (Inland)</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
+      <c r="J5" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t>DS</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -894,12 +903,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="P5" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -912,58 +921,58 @@
           <t>Lager DE – WE Österreich (ig. Lieferung)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr"/>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
         <is>
           <t>ATxxx</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="9" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="M6" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -973,12 +982,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="O6" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="P6" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -991,58 +1000,58 @@
           <t>Lager AT – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1052,12 +1061,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="O7" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="P7" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1070,58 +1079,58 @@
           <t>Lager AT – WE Liechtenstein (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr"/>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K8" s="3" t="inlineStr">
+      <c r="K8" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1131,12 +1140,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr">
+      <c r="O8" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P8" s="3" t="inlineStr">
+      <c r="P8" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1149,58 +1158,58 @@
           <t>Lager DE – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr"/>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L9" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="M9" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1210,12 +1219,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O9" s="3" t="inlineStr">
+      <c r="O9" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="P9" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1228,58 +1237,58 @@
           <t>Konsi-Lager CH – WE Schweiz (CH-Inland)</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>‹Werk CH›</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="J10" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K10" s="3" t="inlineStr">
+      <c r="K10" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L10" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="M10" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1289,12 +1298,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="O10" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="P10" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1307,58 +1316,58 @@
           <t>Konsi-Lager CH – WE Liechtenstein (Schweizer MWST-Raum)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>‹Werk CH›</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr"/>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
+      <c r="J11" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L11" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="M11" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1368,12 +1377,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="O11" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="P11" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -1386,58 +1395,58 @@
           <t>Strecke – Lieferant DE/EU – WE Österreich</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr"/>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>ATxxx</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L12" s="9" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="M12" s="3" t="inlineStr">
+      <c r="M12" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1447,12 +1456,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr">
+      <c r="O12" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P12" s="3" t="inlineStr">
+      <c r="P12" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1465,58 +1474,58 @@
           <t>Strecke – Lieferant DE/EU (≠DE) – WE Deutschland</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr"/>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J13" s="3" t="inlineStr">
+      <c r="J13" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K13" s="3" t="inlineStr">
+      <c r="K13" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L13" s="9" t="inlineStr">
         <is>
           <t>DS</t>
         </is>
       </c>
-      <c r="M13" s="3" t="inlineStr">
+      <c r="M13" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -1526,12 +1535,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr">
+      <c r="O13" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="P13" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1544,58 +1553,58 @@
           <t>Strecke – Lieferant EU – WE Italien (Dreieck, BUKRS AT)</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -1605,12 +1614,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="P14" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1627,58 +1636,58 @@
           <t>Strecke – Lieferant EU – WE Ungarn (Dreieck, BUKRS AT)</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr"/>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="8" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>HUxxx</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L15" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="M15" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -1688,12 +1697,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O15" s="3" t="inlineStr">
+      <c r="O15" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="P15" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1710,58 +1719,58 @@
           <t>Strecke – Lieferant DE – WE Schweiz (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr"/>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E16" s="8" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="H16" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J16" s="3" t="inlineStr">
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="L16" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="M16" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1771,12 +1780,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="O16" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="P16" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1793,58 +1802,58 @@
           <t>Strecke – Lieferant AT – WE Liechtenstein (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr"/>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I17" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J17" s="3" t="inlineStr">
+      <c r="H17" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L17" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="M17" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -1854,12 +1863,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O17" s="3" t="inlineStr">
+      <c r="O17" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P17" s="3" t="inlineStr">
+      <c r="P17" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1876,22 +1885,22 @@
           <t>Strecke EXW – Lieferant AT – WE Deutschland</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -1901,37 +1910,37 @@
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="H18" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="L18" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="M18" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -1941,12 +1950,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O18" s="3" t="inlineStr">
+      <c r="O18" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="P18" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -1959,22 +1968,22 @@
           <t>Strecke EXW – Lieferant DE – WE Italien</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -1984,37 +1993,37 @@
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H19" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I19" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J19" s="3" t="inlineStr">
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L19" s="9" t="inlineStr">
         <is>
           <t>DH</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="M19" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -2024,12 +2033,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O19" s="3" t="inlineStr">
+      <c r="O19" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P19" s="3" t="inlineStr">
+      <c r="P19" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2042,22 +2051,22 @@
           <t>Strecke EXW – Lieferant DE – WE Deutschland (Inland)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2067,37 +2076,37 @@
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H20" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I20" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J20" s="3" t="inlineStr">
+      <c r="J20" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" s="8" t="inlineStr">
         <is>
           <t>DExxx</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L20" s="9" t="inlineStr">
         <is>
           <t>DS</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr">
+      <c r="M20" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -2107,12 +2116,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr">
+      <c r="O20" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P20" s="3" t="inlineStr">
+      <c r="P20" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2125,22 +2134,22 @@
           <t>Strecke EXW – Lieferant IT (ohne EPROHA-Reg) – WE Slowenien</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
         <is>
           <t>EXW</t>
         </is>
@@ -2150,37 +2159,37 @@
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>EXW: Lieferantland -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="H21" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J21" s="8" t="inlineStr">
         <is>
           <t>SI</t>
         </is>
       </c>
-      <c r="K21" s="3" t="inlineStr">
+      <c r="K21" s="8" t="inlineStr">
         <is>
           <t>SIxxx</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="L21" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr">
+      <c r="M21" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -2190,12 +2199,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O21" s="3" t="inlineStr">
+      <c r="O21" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P21" s="3" t="inlineStr">
+      <c r="P21" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2212,58 +2221,58 @@
           <t>Ausfuhr AT → CH (DAP/EXW, Kunde verzollt)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K22" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L22" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="M22" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2273,12 +2282,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O22" s="3" t="inlineStr">
+      <c r="O22" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="P22" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2295,58 +2304,58 @@
           <t>Ausfuhr AT → LI (DAP/EXW, Kunde verzollt)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E23" s="8" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K23" s="3" t="inlineStr">
+      <c r="K23" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="L23" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="M23" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2356,12 +2365,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O23" s="3" t="inlineStr">
+      <c r="O23" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P23" s="3" t="inlineStr">
+      <c r="P23" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2378,58 +2387,58 @@
           <t>Ausfuhr DE → CH (über DE-Reg)</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="8" t="inlineStr">
         <is>
           <t>Ship-to</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
+      <c r="H24" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
+      <c r="I24" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J24" s="3" t="inlineStr">
+      <c r="J24" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K24" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L24" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="M24" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2439,12 +2448,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O24" s="3" t="inlineStr">
+      <c r="O24" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="P24" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2461,58 +2470,58 @@
           <t>CH-Inland DDP – EPROHA CH-registriert – WE Schweiz</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr"/>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>CH-Reg (CH+LI)</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="J25" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K25" s="8" t="inlineStr">
         <is>
           <t>CHxxx</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L25" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="M25" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -2522,12 +2531,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O25" s="3" t="inlineStr">
+      <c r="O25" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="P25" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2544,58 +2553,58 @@
           <t>CH-Reg → WE Liechtenstein (Schweizer MWST-Raum, DDP)</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr"/>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" s="8" t="inlineStr">
         <is>
           <t>CH-Reg (CH+LI)</t>
         </is>
       </c>
-      <c r="H26" s="3" t="inlineStr">
+      <c r="H26" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I26" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="J26" s="3" t="inlineStr">
+      <c r="J26" s="8" t="inlineStr">
         <is>
           <t>LI</t>
         </is>
       </c>
-      <c r="K26" s="3" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
         <is>
           <t>LIxxx</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L26" s="9" t="inlineStr">
         <is>
           <t>B5</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr">
+      <c r="M26" s="8" t="inlineStr">
         <is>
           <t>Inland/CH-Inland</t>
         </is>
@@ -2605,12 +2614,12 @@
           <t>✔ im Code (LI seit PR #75 wie CH)</t>
         </is>
       </c>
-      <c r="O26" s="3" t="inlineStr">
+      <c r="O26" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P26" s="3" t="inlineStr">
+      <c r="P26" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2627,58 +2636,58 @@
           <t>Ausfuhr AT → GB (DAP/EXW, Post-Brexit)</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E27" s="3" t="inlineStr"/>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E27" s="8" t="inlineStr"/>
       <c r="F27" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I27" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J27" s="3" t="inlineStr">
+      <c r="H27" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I27" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J27" s="8" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K27" s="3" t="inlineStr">
+      <c r="K27" s="8" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="L27" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr">
+      <c r="M27" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2688,12 +2697,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O27" s="3" t="inlineStr">
+      <c r="O27" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P27" s="3" t="inlineStr">
+      <c r="P27" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2710,58 +2719,58 @@
           <t>Lager AT – WE Großbritannien (Ausfuhr)</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr"/>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
+      <c r="H28" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K28" s="8" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L28" s="9" t="inlineStr">
         <is>
           <t>A0</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="M28" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2771,12 +2780,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr">
+      <c r="O28" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="P28" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -2789,58 +2798,58 @@
           <t>Lager DE – WE Großbritannien (Ausfuhr über DE-Reg)</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" s="8" t="inlineStr">
         <is>
           <t>‹Werk DE›</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E29" s="3" t="inlineStr"/>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr"/>
       <c r="F29" s="2" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" s="8" t="inlineStr">
         <is>
           <t>Werk</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="H29" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I29" s="3" t="inlineStr">
+      <c r="I29" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="J29" s="3" t="inlineStr">
+      <c r="J29" s="8" t="inlineStr">
         <is>
           <t>GB</t>
         </is>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K29" s="8" t="inlineStr">
         <is>
           <t>GBxxx</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L29" s="9" t="inlineStr">
         <is>
           <t>D0</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="M29" s="8" t="inlineStr">
         <is>
           <t>Ausfuhr Drittland</t>
         </is>
@@ -2850,12 +2859,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr">
+      <c r="O29" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P29" s="3" t="inlineStr">
+      <c r="P29" s="8" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
@@ -2868,58 +2877,58 @@
           <t>Dreieck – Lieferant Deutschland → EPROHA(AT) → WE Italien (Art. 141)</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E30" s="3" t="inlineStr"/>
+      <c r="D30" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E30" s="8" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K30" s="3" t="inlineStr">
+      <c r="K30" s="8" t="inlineStr">
         <is>
           <t>ITxxx</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L30" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="M30" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -2929,12 +2938,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr">
+      <c r="O30" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="P30" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -2951,58 +2960,58 @@
           <t>Dreieck – Lieferant Frankreich → EPROHA(AT) → WE Ungarn (Art. 141)</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr"/>
+      <c r="D31" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E31" s="8" t="inlineStr"/>
       <c r="F31" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>Ship-to -&gt; BUKRS AT</t>
         </is>
       </c>
-      <c r="H31" s="3" t="inlineStr">
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="I31" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="I31" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J31" s="8" t="inlineStr">
         <is>
           <t>HU</t>
         </is>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="K31" s="8" t="inlineStr">
         <is>
           <t>HUxxx</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L31" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="M31" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -3012,12 +3021,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O31" s="3" t="inlineStr">
+      <c r="O31" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P31" s="3" t="inlineStr">
+      <c r="P31" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3034,58 +3043,58 @@
           <t>Drop-Ship – Kunde AT (legt fremde EU-UID vor) – Warenempfänger DE</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr"/>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="8" t="inlineStr">
         <is>
           <t>Kunde-UID (≠AT)</t>
         </is>
       </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K32" s="8" t="inlineStr">
         <is>
           <t>DE(Kunde AT)xxx</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L32" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="M32" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung</t>
         </is>
@@ -3095,12 +3104,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O32" s="3" t="inlineStr">
+      <c r="O32" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P32" s="3" t="inlineStr">
+      <c r="P32" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3117,58 +3126,58 @@
           <t>Drop-Ship – Kunde AT (KEINE fremde UID) – Warenempfänger DE</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr"/>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr"/>
       <c r="F33" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="8" t="inlineStr">
         <is>
           <t>BUKRS AT</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I33" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J33" s="3" t="inlineStr">
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="K33" s="8" t="inlineStr">
         <is>
           <t>DE(Kunde AT)xxx</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L33" s="9" t="inlineStr">
         <is>
           <t>A2</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr">
+      <c r="M33" s="8" t="inlineStr">
         <is>
           <t>Inland AT 20%</t>
         </is>
@@ -3178,12 +3187,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O33" s="3" t="inlineStr">
+      <c r="O33" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P33" s="3" t="inlineStr">
+      <c r="P33" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3200,58 +3209,58 @@
           <t>Drop-Ship – Kunde DE – Warenempfänger IT (Reihen-/Dreiecksgeschäft)</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr"/>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="8" t="inlineStr">
         <is>
           <t>AT (Ansässigkeit)</t>
         </is>
       </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K34" s="8" t="inlineStr">
         <is>
           <t>DE(Kunde)xxx</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="L34" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="M34" s="8" t="inlineStr">
         <is>
           <t>ig. Lieferung / Dreieck</t>
         </is>
@@ -3261,12 +3270,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O34" s="3" t="inlineStr">
+      <c r="O34" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P34" s="3" t="inlineStr">
+      <c r="P34" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3283,58 +3292,58 @@
           <t>Drop-Ship – Kunde CH (Drittland) – Warenempfänger SK (Ware bleibt EU)</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>EPROHA ‹Nr.›</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>‹Werk AT›</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr"/>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>AT (Ansässigkeit)</t>
         </is>
       </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="I35" s="3" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="J35" s="3" t="inlineStr">
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
         <is>
           <t>SK</t>
         </is>
       </c>
-      <c r="K35" s="3" t="inlineStr">
+      <c r="K35" s="8" t="inlineStr">
         <is>
           <t>CH(Kunde)xxx</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L35" s="9" t="inlineStr">
         <is>
           <t>AF</t>
         </is>
       </c>
-      <c r="M35" s="3" t="inlineStr">
+      <c r="M35" s="8" t="inlineStr">
         <is>
           <t>ig. Reihengeschäft (kein Export)</t>
         </is>
@@ -3344,12 +3353,12 @@
           <t>✔ im Code</t>
         </is>
       </c>
-      <c r="O35" s="3" t="inlineStr">
+      <c r="O35" s="8" t="inlineStr">
         <is>
           <t>Unsere UID lautet: xxx</t>
         </is>
       </c>
-      <c r="P35" s="3" t="inlineStr">
+      <c r="P35" s="8" t="inlineStr">
         <is>
           <t>⟶ in SAP prüfen</t>
         </is>
@@ -3473,7 +3482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -3540,37 +3549,37 @@
           <t>Lieferant DE → Ware nach AT</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>bewegt</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>VE</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>ig. Erwerb (Selbstveranlagung)</t>
         </is>
@@ -3587,37 +3596,37 @@
           <t>Lieferant IT → Ware nach AT</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C3" s="8" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>bewegt</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="12" t="inlineStr">
         <is>
           <t>VE</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>ig. Erwerb (Selbstveranlagung)</t>
         </is>
@@ -3634,37 +3643,37 @@
           <t>Lieferant FR → Ware nach DE (wir DE-registriert)</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>FR</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>bewegt</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="11" t="inlineStr">
         <is>
           <t>DE248554278</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>VH</t>
         </is>
       </c>
-      <c r="H4" s="8" t="inlineStr">
+      <c r="H4" s="11" t="inlineStr">
         <is>
           <t>ig. Erwerb (Selbstveranlagung)</t>
         </is>
@@ -3681,37 +3690,37 @@
           <t>Lieferant AT → AT-Inlandslieferung an uns</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>ruhend</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>ATU36513402</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="12" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="H5" s="8" t="inlineStr">
+      <c r="H5" s="11" t="inlineStr">
         <is>
           <t>Inlandseinkauf (Vorsteuer)</t>
         </is>
@@ -3725,327 +3734,374 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Lieferant DE → DE-Inlandslieferung an uns</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
+          <t>EXW-Strecke: Lieferant AT → EPROHA, danach ig. Lieferung AT→DE (Verkauf AF)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>ruhend</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>DE248554278</t>
-        </is>
-      </c>
-      <c r="G6" s="9" t="inlineStr">
-        <is>
-          <t>VD</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>ATU36513402</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>Inlandseinkauf (Vorsteuer)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>19% DE-Vorsteuer VD</t>
+          <t>Vorlieferung RUHEND in AT (EPROHAs Verkauf AT→DE ist die bewegte Lieferung AF); AT-Lieferant weist 20% AT-MwSt aus → Vorsteuer V2. Verknüpft mit Verkaufszeile „Strecke EXW – Lieferant AT – WE Deutschland“.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Lieferant CH → CH-Inlandslieferung (wir CH-registriert)</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
+          <t>Lieferant DE → DE-Inlandslieferung an uns</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>ruhend</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>CHE-113.857.016 MWST</t>
-        </is>
-      </c>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>IB</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>DE248554278</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>VD</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
         <is>
           <t>Inlandseinkauf (Vorsteuer)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>8,1% CH-Vorsteuer IB</t>
+          <t>19% DE-Vorsteuer VD</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lieferant LI → LI-Inlandslieferung (Schweizer MWST-Raum)</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
+          <t>Lieferant CH → CH-Inlandslieferung (wir CH-registriert)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>LI</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>ruhend</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>LI</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
         <is>
           <t>CHE-113.857.016 MWST</t>
         </is>
       </c>
-      <c r="G8" s="9" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr">
         <is>
           <t>IB</t>
         </is>
       </c>
-      <c r="H8" s="8" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>Inlandseinkauf (Vorsteuer)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>8,1% Vorsteuer IB – LI über CH-Registrierung</t>
+          <t>8,1% CH-Vorsteuer IB</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>AT Werklieferung/Leistung mit Reverse Charge</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
+          <t>Lieferant LI → LI-Inlandslieferung (Schweizer MWST-Raum)</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>ruhend</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>ATU36513402</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>RC</t>
-        </is>
-      </c>
-      <c r="H9" s="8" t="inlineStr">
-        <is>
-          <t>Reverse Charge</t>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>LI</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>CHE-113.857.016 MWST</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>IB</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Inlandseinkauf (Vorsteuer)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>AT-RC (§19 UStG) → Eingang RC</t>
+          <t>8,1% Vorsteuer IB – LI über CH-Registrierung</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lieferant CH → Einfuhr nach AT</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
+          <t>AT Werklieferung/Leistung mit Reverse Charge</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>CH</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Einfuhr</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>EORI (keine UID)</t>
-        </is>
-      </c>
-      <c r="G10" s="10" t="inlineStr">
-        <is>
-          <t>EUSt / EORI (kein MWSKZ)</t>
-        </is>
-      </c>
-      <c r="H10" s="8" t="inlineStr">
-        <is>
-          <t>Einfuhr Drittland</t>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>ruhend</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>ATU36513402</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>RC</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>Reverse Charge</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>EUSt über EORI, als Vorsteuer abziehbar – kein Tabellen-MWSKZ</t>
+          <t>AT-RC (§19 UStG) → Eingang RC</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Lieferant GB → Einfuhr nach AT</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
+          <t>Lieferant CH → Einfuhr nach AT</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>GB</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>Einfuhr</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
         <is>
           <t>EORI (keine UID)</t>
         </is>
       </c>
-      <c r="G11" s="10" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>EUSt / EORI (kein MWSKZ)</t>
         </is>
       </c>
-      <c r="H11" s="8" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>Einfuhr Drittland</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>EUSt über EORI (Post-Brexit)</t>
+          <t>EUSt über EORI, als Vorsteuer abziehbar – kein Tabellen-MWSKZ</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Lieferant GB → Einfuhr nach AT</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>EPROHA</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Einfuhr</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>EORI (keine UID)</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>EUSt / EORI (kein MWSKZ)</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Einfuhr Drittland</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>EUSt über EORI (Post-Brexit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Eigene Ware ab AT-Lager (Direktlieferung)</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>EPROHA</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>entfällt</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>AT</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>AT</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="G12" s="10" t="inlineStr">
+      <c r="G13" s="13" t="inlineStr">
         <is>
           <t>not relevant</t>
         </is>
       </c>
-      <c r="H12" s="8" t="inlineStr">
+      <c r="H13" s="11" t="inlineStr">
         <is>
           <t>kein Vorsteuervorgang</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>kein Vorsteuervorgang</t>
         </is>

</xml_diff>